<commit_message>
add: finalizing on ctc
</commit_message>
<xml_diff>
--- a/Data/Clean_KDHS_GBV_Data_By_County.xlsx
+++ b/Data/Clean_KDHS_GBV_Data_By_County.xlsx
@@ -25,7 +25,7 @@
     <t>%Physical_Violence_12mo_pct (29C)</t>
   </si>
   <si>
-    <t>%Sexual_Violence_ever_pct (31C)</t>
+    <t>%Sexual_Violence_12mo_pct (31C)</t>
   </si>
   <si>
     <t>Number_of_Women</t>
@@ -642,7 +642,7 @@
   <cols>
     <col min="1" max="1" style="17" width="18.576428571428572" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="18" width="46.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="18" width="43.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="18" width="45.14785714285715" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="19" width="25.290714285714284" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="17" width="9.147857142857141" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
@@ -660,7 +660,7 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="24.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="23.25">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -685,7 +685,7 @@
         <v>11.5</v>
       </c>
       <c r="C3" s="9">
-        <v>9.8</v>
+        <v>3.8</v>
       </c>
       <c r="D3" s="10">
         <v>500</v>
@@ -702,7 +702,7 @@
         <v>11.3</v>
       </c>
       <c r="C4" s="9">
-        <v>4.3</v>
+        <v>3.3</v>
       </c>
       <c r="D4" s="10">
         <v>264</v>
@@ -719,7 +719,7 @@
         <v>8.3</v>
       </c>
       <c r="C5" s="9">
-        <v>12.2</v>
+        <v>6.5</v>
       </c>
       <c r="D5" s="10">
         <v>491</v>
@@ -736,7 +736,7 @@
         <v>23.2</v>
       </c>
       <c r="C6" s="9">
-        <v>2.3</v>
+        <v>1.5</v>
       </c>
       <c r="D6" s="10">
         <v>81</v>
@@ -753,7 +753,7 @@
         <v>12</v>
       </c>
       <c r="C7" s="9">
-        <v>14.5</v>
+        <v>6.3</v>
       </c>
       <c r="D7" s="10">
         <v>51</v>
@@ -770,7 +770,7 @@
         <v>7.4</v>
       </c>
       <c r="C8" s="9">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="D8" s="10">
         <v>110</v>
@@ -787,7 +787,7 @@
         <v>12.8</v>
       </c>
       <c r="C9" s="9">
-        <v>5.8</v>
+        <v>3.5</v>
       </c>
       <c r="D9" s="10">
         <v>148</v>
@@ -804,7 +804,7 @@
         <v>5.5</v>
       </c>
       <c r="C10" s="9">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="D10" s="10">
         <v>84</v>
@@ -855,7 +855,7 @@
         <v>29.3</v>
       </c>
       <c r="C13" s="9">
-        <v>9.2</v>
+        <v>5.3</v>
       </c>
       <c r="D13" s="10">
         <v>69</v>
@@ -872,7 +872,7 @@
         <v>15.1</v>
       </c>
       <c r="C14" s="9">
-        <v>16</v>
+        <v>8.2</v>
       </c>
       <c r="D14" s="10">
         <v>547</v>
@@ -889,7 +889,7 @@
         <v>13.9</v>
       </c>
       <c r="C15" s="9">
-        <v>12.5</v>
+        <v>6.9</v>
       </c>
       <c r="D15" s="10">
         <v>146</v>
@@ -906,7 +906,7 @@
         <v>27.7</v>
       </c>
       <c r="C16" s="9">
-        <v>21.5</v>
+        <v>13</v>
       </c>
       <c r="D16" s="10">
         <v>207</v>
@@ -923,7 +923,7 @@
         <v>4.7</v>
       </c>
       <c r="C17" s="9">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="D17" s="10">
         <v>391</v>
@@ -940,7 +940,7 @@
         <v>10.1</v>
       </c>
       <c r="C18" s="9">
-        <v>6.3</v>
+        <v>3</v>
       </c>
       <c r="D18" s="10">
         <v>515</v>
@@ -957,7 +957,7 @@
         <v>11.9</v>
       </c>
       <c r="C19" s="9">
-        <v>4.7</v>
+        <v>3.2</v>
       </c>
       <c r="D19" s="10">
         <v>362</v>
@@ -974,7 +974,7 @@
         <v>5</v>
       </c>
       <c r="C20" s="9">
-        <v>17.5</v>
+        <v>6.9</v>
       </c>
       <c r="D20" s="10">
         <v>222</v>
@@ -991,7 +991,7 @@
         <v>15.4</v>
       </c>
       <c r="C21" s="9">
-        <v>15.1</v>
+        <v>5.6</v>
       </c>
       <c r="D21" s="10">
         <v>276</v>
@@ -1008,7 +1008,7 @@
         <v>12.5</v>
       </c>
       <c r="C22" s="9">
-        <v>12.9</v>
+        <v>3.2</v>
       </c>
       <c r="D22" s="10">
         <v>263</v>
@@ -1025,7 +1025,7 @@
         <v>22</v>
       </c>
       <c r="C23" s="9">
-        <v>24.3</v>
+        <v>13.6</v>
       </c>
       <c r="D23" s="10">
         <v>359</v>
@@ -1042,7 +1042,7 @@
         <v>17.9</v>
       </c>
       <c r="C24" s="9">
-        <v>16.6</v>
+        <v>9.8</v>
       </c>
       <c r="D24" s="10">
         <v>1091</v>
@@ -1059,7 +1059,7 @@
         <v>19.9</v>
       </c>
       <c r="C25" s="9">
-        <v>10.8</v>
+        <v>6.7</v>
       </c>
       <c r="D25" s="10">
         <v>176</v>
@@ -1076,7 +1076,7 @@
         <v>19.1</v>
       </c>
       <c r="C26" s="9">
-        <v>7.5</v>
+        <v>6.3</v>
       </c>
       <c r="D26" s="10">
         <v>205</v>
@@ -1093,7 +1093,7 @@
         <v>28.5</v>
       </c>
       <c r="C27" s="9">
-        <v>6.9</v>
+        <v>4.2</v>
       </c>
       <c r="D27" s="10">
         <v>87</v>
@@ -1110,7 +1110,7 @@
         <v>17.2</v>
       </c>
       <c r="C28" s="9">
-        <v>13.1</v>
+        <v>5.6</v>
       </c>
       <c r="D28" s="10">
         <v>351</v>
@@ -1127,7 +1127,7 @@
         <v>12.4</v>
       </c>
       <c r="C29" s="9">
-        <v>9.9</v>
+        <v>4.6</v>
       </c>
       <c r="D29" s="10">
         <v>495</v>
@@ -1144,7 +1144,7 @@
         <v>15.9</v>
       </c>
       <c r="C30" s="9">
-        <v>6.9</v>
+        <v>4</v>
       </c>
       <c r="D30" s="10">
         <v>119</v>
@@ -1161,7 +1161,7 @@
         <v>15</v>
       </c>
       <c r="C31" s="9">
-        <v>6</v>
+        <v>2.6</v>
       </c>
       <c r="D31" s="10">
         <v>334</v>
@@ -1178,7 +1178,7 @@
         <v>19.6</v>
       </c>
       <c r="C32" s="9">
-        <v>8.4</v>
+        <v>5.7</v>
       </c>
       <c r="D32" s="10">
         <v>207</v>
@@ -1195,7 +1195,7 @@
         <v>11.7</v>
       </c>
       <c r="C33" s="9">
-        <v>10.9</v>
+        <v>3.1</v>
       </c>
       <c r="D33" s="10">
         <v>175</v>
@@ -1212,7 +1212,7 @@
         <v>9.4</v>
       </c>
       <c r="C34" s="9">
-        <v>13.8</v>
+        <v>3.6</v>
       </c>
       <c r="D34" s="10">
         <v>898</v>
@@ -1229,7 +1229,7 @@
         <v>16.3</v>
       </c>
       <c r="C35" s="9">
-        <v>17.5</v>
+        <v>8.7</v>
       </c>
       <c r="D35" s="10">
         <v>376</v>
@@ -1246,7 +1246,7 @@
         <v>17</v>
       </c>
       <c r="C36" s="9">
-        <v>16.9</v>
+        <v>8.6</v>
       </c>
       <c r="D36" s="10">
         <v>471</v>
@@ -1263,7 +1263,7 @@
         <v>10.2</v>
       </c>
       <c r="C37" s="9">
-        <v>3.2</v>
+        <v>1.5</v>
       </c>
       <c r="D37" s="10">
         <v>386</v>
@@ -1280,7 +1280,7 @@
         <v>10.7</v>
       </c>
       <c r="C38" s="9">
-        <v>12.9</v>
+        <v>7.4</v>
       </c>
       <c r="D38" s="10">
         <v>369</v>
@@ -1297,7 +1297,7 @@
         <v>19.1</v>
       </c>
       <c r="C39" s="9">
-        <v>16.8</v>
+        <v>8.9</v>
       </c>
       <c r="D39" s="10">
         <v>707</v>
@@ -1314,7 +1314,7 @@
         <v>17.1</v>
       </c>
       <c r="C40" s="9">
-        <v>11.9</v>
+        <v>5.6</v>
       </c>
       <c r="D40" s="10">
         <v>195</v>
@@ -1331,7 +1331,7 @@
         <v>29.4</v>
       </c>
       <c r="C41" s="9">
-        <v>30.3</v>
+        <v>16.6</v>
       </c>
       <c r="D41" s="10">
         <v>623</v>
@@ -1348,7 +1348,7 @@
         <v>21.1</v>
       </c>
       <c r="C42" s="9">
-        <v>14.7</v>
+        <v>8.9</v>
       </c>
       <c r="D42" s="10">
         <v>309</v>
@@ -1365,7 +1365,7 @@
         <v>16.9</v>
       </c>
       <c r="C43" s="9">
-        <v>5.7</v>
+        <v>4.3</v>
       </c>
       <c r="D43" s="10">
         <v>291</v>
@@ -1382,7 +1382,7 @@
         <v>26</v>
       </c>
       <c r="C44" s="9">
-        <v>10.8</v>
+        <v>6.6</v>
       </c>
       <c r="D44" s="10">
         <v>420</v>
@@ -1399,7 +1399,7 @@
         <v>26.6</v>
       </c>
       <c r="C45" s="9">
-        <v>23.1</v>
+        <v>10.8</v>
       </c>
       <c r="D45" s="10">
         <v>352</v>
@@ -1416,7 +1416,7 @@
         <v>29.5</v>
       </c>
       <c r="C46" s="9">
-        <v>16.7</v>
+        <v>7.4</v>
       </c>
       <c r="D46" s="10">
         <v>364</v>
@@ -1433,7 +1433,7 @@
         <v>19.8</v>
       </c>
       <c r="C47" s="9">
-        <v>16</v>
+        <v>10.1</v>
       </c>
       <c r="D47" s="10">
         <v>404</v>
@@ -1450,7 +1450,7 @@
         <v>11.3</v>
       </c>
       <c r="C48" s="9">
-        <v>14.5</v>
+        <v>6.3</v>
       </c>
       <c r="D48" s="10">
         <v>176</v>
@@ -1467,7 +1467,7 @@
         <v>13.5</v>
       </c>
       <c r="C49" s="9">
-        <v>12.2</v>
+        <v>5.8</v>
       </c>
       <c r="D49" s="10">
         <v>2088</v>
@@ -1484,7 +1484,7 @@
         <v>15.8</v>
       </c>
       <c r="C50" s="12">
-        <v>13</v>
+        <v>6.5</v>
       </c>
       <c r="D50" s="13">
         <v>16926</v>

</xml_diff>